<commit_message>
Semaine 2 : AMDEC : échelles + 17 modes, actions préconisées et cotations
</commit_message>
<xml_diff>
--- a/sdf-etude-de-cas/AMDEC_alim_secours.xlsx
+++ b/sdf-etude-de-cas/AMDEC_alim_secours.xlsx
@@ -7,14 +7,14 @@
   </bookViews>
   <sheets>
     <sheet name="échelles" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="AMDEC" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="131">
   <si>
     <t>Effets Jeu de Barre</t>
   </si>
@@ -94,6 +94,12 @@
     <t>Détection inefficace</t>
   </si>
   <si>
+    <t>Autonomie Batterie Onduleur (en heures)</t>
+  </si>
+  <si>
+    <t>charges critiques : aucune coupure tolérée</t>
+  </si>
+  <si>
     <t>N°</t>
   </si>
   <si>
@@ -145,157 +151,262 @@
     <t>IPR'</t>
   </si>
   <si>
+    <t>GE1+GE2 (DCC)</t>
+  </si>
+  <si>
+    <t>produire la puissance requise à tension et fréquence nominales pendant 24 h</t>
+  </si>
+  <si>
+    <t>arrêt en fonctionnement simultané</t>
+  </si>
+  <si>
+    <t>carburant pollué → colmatage filtres</t>
+  </si>
+  <si>
+    <t>GE1 et GE2 s'arrête en cours de mission</t>
+  </si>
+  <si>
+    <t>perte totale de l'alimentation après décharge des batteries</t>
+  </si>
+  <si>
+    <t>analyse périodique du carburant</t>
+  </si>
+  <si>
+    <t>analyse et rotation du carburant</t>
+  </si>
+  <si>
+    <t>Jeu de barres</t>
+  </si>
+  <si>
+    <t>distribuer l’énergie vers les départs des charges critiques</t>
+  </si>
+  <si>
+    <t>défaut d'isolement</t>
+  </si>
+  <si>
+    <t>contamination de surface (poussière...)</t>
+  </si>
+  <si>
+    <t>isolation défaillante</t>
+  </si>
+  <si>
+    <t>perte totale de l’alimentation</t>
+  </si>
+  <si>
+    <t>thermographie infrarouge + contrôle isolement</t>
+  </si>
+  <si>
+    <t>Onduleur</t>
+  </si>
+  <si>
+    <t>assurer l’autonomie (batteries) pendant le démarrage des GE et la commutation</t>
+  </si>
+  <si>
+    <t>autonomie insuffisante</t>
+  </si>
+  <si>
+    <t>vieillissement des batteries (capacité réduite)</t>
+  </si>
+  <si>
+    <t>batteries indisponibles à la sollicitation</t>
+  </si>
+  <si>
+    <t>coupure brève du jeu de barres jusqu’à la reprise par le GE</t>
+  </si>
+  <si>
+    <t>essai périodique d'autonomie + alarme onduleur</t>
+  </si>
+  <si>
+    <t>remplacement préventif selon l’âge + essai d’autonomie</t>
+  </si>
+  <si>
+    <t>fournir aux charges une tension alternative stable et sans coupure</t>
+  </si>
+  <si>
+    <t>perte de sortie onduleur</t>
+  </si>
+  <si>
+    <t>surchauffe (ventilation)</t>
+  </si>
+  <si>
+    <t>onduleur hors service</t>
+  </si>
+  <si>
+    <t>bascule sur bypass statique : jeu de barres alimenté mais plus protégé contre les coupures</t>
+  </si>
+  <si>
+    <t>alarme onduleur / surveillance température</t>
+  </si>
+  <si>
+    <t>Inverseur</t>
+  </si>
+  <si>
+    <t>détecter/commuter et conduire le courant</t>
+  </si>
+  <si>
+    <t>retour intempestif entre les deux sources</t>
+  </si>
+  <si>
+    <t>seuils trop sensibles</t>
+  </si>
+  <si>
+    <t>la bascule s'effectue même lorsque le réseau n'est pas revenu</t>
+  </si>
+  <si>
+    <t>jeu de barres alimenté par l’onduleur sur batteries ; risque de pompage → décharge progressive des batteries</t>
+  </si>
+  <si>
+    <t>panneau de commande + essai périodique</t>
+  </si>
+  <si>
+    <t>vérification des seuils et temporisations à la mise en service et à chaque essai</t>
+  </si>
+  <si>
+    <t>maintenir la position/conduire le courant</t>
+  </si>
+  <si>
+    <t>courant mal conduit</t>
+  </si>
+  <si>
+    <t>contacts usés -&gt; échauffement</t>
+  </si>
+  <si>
+    <t>échauffement anormal des contacts</t>
+  </si>
+  <si>
+    <t>état dégradé</t>
+  </si>
+  <si>
+    <t>thermographie infrarouge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">commutation non maintenue  </t>
+  </si>
+  <si>
+    <t>fusible de commande endommagé</t>
+  </si>
+  <si>
+    <t>bobine retombe</t>
+  </si>
+  <si>
+    <t>perte totale de l'alimentation après autonomie des batteries</t>
+  </si>
+  <si>
+    <t>surveillance de la tension de commande + alarme</t>
+  </si>
+  <si>
+    <t>détecter la perte du réseau et commuter sur la source de secours (dans un délai donné)</t>
+  </si>
+  <si>
+    <t>commutation effectuée même sans perte de réseau</t>
+  </si>
+  <si>
+    <t>la bascule s'effectue même lorsqu'il n'y a pas de perte de réseau effective</t>
+  </si>
+  <si>
+    <t>effet intempestif, basculement inutile, décharge des batteries et consommation de carburant</t>
+  </si>
+  <si>
+    <t>commutation trop lente</t>
+  </si>
+  <si>
+    <t>relais fatigués</t>
+  </si>
+  <si>
+    <t>la détection de perte est trop lente</t>
+  </si>
+  <si>
+    <t>décharge des batteries plus prononcée</t>
+  </si>
+  <si>
+    <t>essai périodique (mesure du temps de commutation contre la valeur attendue (Autonomie Batterie Onduleur))</t>
+  </si>
+  <si>
+    <t>commutation non effectuée</t>
+  </si>
+  <si>
+    <t>sélecteur en mauvaise position</t>
+  </si>
+  <si>
+    <t>La bascule ne s'effectue pas</t>
+  </si>
+  <si>
+    <t>perte totale de l'alimentation</t>
+  </si>
+  <si>
     <t>GE1/GE2</t>
   </si>
   <si>
+    <t>puissance trop faible constatée</t>
+  </si>
+  <si>
+    <t>problème moteur</t>
+  </si>
+  <si>
+    <t>GE délivre une puissance réduite</t>
+  </si>
+  <si>
+    <t>état dégradé, redondance dégradée</t>
+  </si>
+  <si>
+    <t>capteurs mesures facteurs pouvant affecter le moteur (mesure puissance / tension / fréquence + alarme)</t>
+  </si>
+  <si>
+    <t>arrêt en fonctionnement</t>
+  </si>
+  <si>
+    <t>manque de carburant</t>
+  </si>
+  <si>
+    <t>GE s'arrête</t>
+  </si>
+  <si>
+    <t>état dégradé, plus de redondance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jauge de carburant + alarme carburant vide + essai périodique mensuel </t>
+  </si>
+  <si>
     <t>démarrer sur sollicitation dans le délai requis</t>
   </si>
   <si>
+    <t>refus de démarrage simultané</t>
+  </si>
+  <si>
+    <t>carburant trop vieux (cuve commune, dégrade les deux GE)</t>
+  </si>
+  <si>
+    <t>GE1 et GE2 ne démarrent pas</t>
+  </si>
+  <si>
+    <t>essai périodique mensuel</t>
+  </si>
+  <si>
     <t>refus de démarrage</t>
   </si>
   <si>
-    <t>manque de carburant</t>
+    <t>robinet d'accès carburant en position OFF</t>
   </si>
   <si>
     <t>GE indisponible à la sollicitation</t>
   </si>
   <si>
-    <t>état dégradé, plus de redondance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jauge de carburant + alarme carburant vide + essai périodique mensuel </t>
+    <t xml:space="preserve">capteur de position + essai périodique mensuel </t>
+  </si>
+  <si>
+    <t>batterie de démarrage déchargée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">surveillance du chargeur / tension batterie de démarrage avec alarme + essai périodique mensuel </t>
+  </si>
+  <si>
+    <t>vérification et recharge périodique des batteries</t>
   </si>
   <si>
     <t>manque d'huile moteur</t>
   </si>
   <si>
     <t xml:space="preserve">jauge d'huile moteur + alarme huile moteur vide + essai périodique mensuel </t>
-  </si>
-  <si>
-    <t>batterie de démarrage déchargée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">surveillance du chargeur / tension batterie de démarrage avec alarme + essai périodique mensuel </t>
-  </si>
-  <si>
-    <t>robinet d'accès carburant en position OFF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">capteur de position + essai périodique mensuel </t>
-  </si>
-  <si>
-    <t>GE1+GE2 (DCC)</t>
-  </si>
-  <si>
-    <t>démarrage trop lent</t>
-  </si>
-  <si>
-    <t>carburant trop vieux (cuve commune, dégrade les deux GE)</t>
-  </si>
-  <si>
-    <t>GE1 et GE2 démarrent, mais dans un temps plus long que spécifié</t>
-  </si>
-  <si>
-    <t>perte totale de l'alimentation après décharge des batteries</t>
-  </si>
-  <si>
-    <t>essai périodique mensuel</t>
-  </si>
-  <si>
-    <t>produire la puissance requise à tension et fréquence nominales pendant 24 h</t>
-  </si>
-  <si>
-    <t>arrêt en fonctionnement</t>
-  </si>
-  <si>
-    <t>GE s'arrête</t>
-  </si>
-  <si>
-    <t>jauge de carburant + alarme carburant vide</t>
-  </si>
-  <si>
-    <t>puissance trop faible constatée</t>
-  </si>
-  <si>
-    <t>problème moteur</t>
-  </si>
-  <si>
-    <t>GE délivre une puissance réduite</t>
-  </si>
-  <si>
-    <t>état dégradé, redondance dégradée</t>
-  </si>
-  <si>
-    <t>capteurs mesures facteurs pouvant affecter le moteur (mesure puissance / tension / fréquence + alarme)</t>
-  </si>
-  <si>
-    <t>Inverseur</t>
-  </si>
-  <si>
-    <t>détecter la perte du réseau et commuter sur la source de secours (dans un délai donné)</t>
-  </si>
-  <si>
-    <t>commutation non effectuée</t>
-  </si>
-  <si>
-    <t>sélecteur en mauvaise position</t>
-  </si>
-  <si>
-    <t>La bascule ne s'effectue pas</t>
-  </si>
-  <si>
-    <t>perte totale de l'alimentation</t>
-  </si>
-  <si>
-    <t>panneau de commande + essai périodique</t>
-  </si>
-  <si>
-    <t>commutation trop lente</t>
-  </si>
-  <si>
-    <t>relais fatigués</t>
-  </si>
-  <si>
-    <t>la détection de perte est trop lente</t>
-  </si>
-  <si>
-    <t>perte totale de l'alimentation, retour après un délai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essai périodique  </t>
-  </si>
-  <si>
-    <t>commutation effectuée même sans perte de réseau</t>
-  </si>
-  <si>
-    <t>seuils trop sensibles</t>
-  </si>
-  <si>
-    <t>la bascule s'effectue même lorsqu'il n'y a pas de perte de réseau effective</t>
-  </si>
-  <si>
-    <t>maintenir la position/conduire le courant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">commutation non maintenue  </t>
-  </si>
-  <si>
-    <t>la bascule s'effectue même lorsque le réseau n'est pas revenu</t>
-  </si>
-  <si>
-    <t>courant mal conduit</t>
-  </si>
-  <si>
-    <t>fusible de commande endommagé</t>
-  </si>
-  <si>
-    <t>perte du courant de controle</t>
-  </si>
-  <si>
-    <t>état dégradé</t>
-  </si>
-  <si>
-    <t>capteur de courant</t>
   </si>
 </sst>
 </file>
@@ -622,6 +733,20 @@
     <row r="8">
       <c r="B8" s="4"/>
     </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9">
+        <f>1/6</f>
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+    </row>
     <row r="16">
       <c r="A16" s="3"/>
     </row>
@@ -657,310 +782,343 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I2" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J2" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K2" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L2" s="1">
         <f>I2*J2*K2</f>
-        <v>60</v>
-      </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
+        <v>160</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="N2" s="2">
+        <v>10</v>
+      </c>
+      <c r="O2" s="2">
+        <v>2</v>
+      </c>
+      <c r="P2" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q2" s="2">
+        <f>N2*O2*P2</f>
+        <v>80</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I3" s="1">
+        <v>10</v>
+      </c>
+      <c r="J3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I3" s="1">
-        <v>5</v>
-      </c>
-      <c r="J3" s="1">
-        <v>5</v>
-      </c>
       <c r="K3" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L3" s="1">
         <f>I3*J3*K3</f>
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
+      <c r="Q3" s="2">
+        <f>N3*O3*P3</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I4" s="1">
+        <v>8</v>
+      </c>
+      <c r="J4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="I4" s="1">
-        <v>5</v>
-      </c>
-      <c r="J4" s="1">
-        <v>7</v>
-      </c>
       <c r="K4" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L4" s="1">
         <f>I4*J4*K4</f>
-        <v>140</v>
-      </c>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
+        <v>144</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="N4" s="2">
+        <v>8</v>
+      </c>
+      <c r="O4" s="2">
+        <v>2</v>
+      </c>
+      <c r="P4" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="2">
+        <f>N4*O4*P4</f>
+        <v>64</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="I5" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J5" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K5" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L5" s="1">
         <f>I5*J5*K5</f>
-        <v>15</v>
+        <v>64</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
+      <c r="Q5" s="2">
+        <f>N5*O5*P5</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I6" s="1">
+        <v>6</v>
+      </c>
+      <c r="J6" s="1">
+        <v>3</v>
+      </c>
+      <c r="K6" s="1">
         <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I6" s="1">
-        <v>10</v>
-      </c>
-      <c r="J6" s="1">
-        <v>4</v>
-      </c>
-      <c r="K6" s="1">
-        <v>9</v>
       </c>
       <c r="L6" s="1">
         <f>I6*J6*K6</f>
-        <v>360</v>
-      </c>
-      <c r="M6" s="2"/>
+        <v>90</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
+      <c r="Q6" s="2">
+        <f>N6*O6*P6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>43</v>
+        <v>74</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>46</v>
+        <v>84</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>64</v>
+        <v>85</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>48</v>
+        <v>86</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="I7" s="1">
         <v>5</v>
       </c>
       <c r="J7" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K7" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L7" s="1">
         <f>I7*J7*K7</f>
@@ -970,35 +1128,38 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
+      <c r="Q7" s="2">
+        <f>N7*O7*P7</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>43</v>
+        <v>74</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="I8" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J8" s="1">
         <v>4</v>
@@ -1008,326 +1169,512 @@
       </c>
       <c r="L8" s="1">
         <f>I8*J8*K8</f>
-        <v>60</v>
-      </c>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
+        <v>200</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="N8" s="2">
+        <v>10</v>
+      </c>
+      <c r="O8" s="2">
+        <v>4</v>
+      </c>
+      <c r="P8" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="2">
+        <f>N8*O8*P8</f>
+        <v>120</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="I9" s="1">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J9" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="1">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L9" s="1">
         <f>I9*J9*K9</f>
-        <v>270</v>
-      </c>
-      <c r="M9" s="2"/>
+        <v>30</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
+      <c r="Q9" s="2">
+        <f>N9*O9*P9</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="I10" s="1">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J10" s="1">
         <v>2</v>
       </c>
       <c r="K10" s="1">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L10" s="1">
         <f>I10*J10*K10</f>
-        <v>162</v>
+        <v>24</v>
       </c>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
+      <c r="Q10" s="2">
+        <f>N10*O10*P10</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
+        <v>8</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="I11" s="1">
+      <c r="J11" s="1">
         <v>3</v>
       </c>
-      <c r="J11" s="1">
-        <v>2</v>
-      </c>
       <c r="K11" s="1">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L11" s="1">
         <f>I11*J11*K11</f>
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
+      <c r="Q11" s="2">
+        <f>N11*O11*P11</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>86</v>
+        <v>46</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>76</v>
+        <v>110</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="I12" s="1">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J12" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K12" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L12" s="1">
         <f>I12*J12*K12</f>
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
+      <c r="Q12" s="2">
+        <f>N12*O12*P12</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>86</v>
+        <v>46</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="I13" s="1">
         <v>5</v>
       </c>
       <c r="J13" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K13" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L13" s="1">
         <f>I13*J13*K13</f>
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
+      <c r="Q13" s="2">
+        <f>N13*O13*P13</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
+      <c r="A14" s="1">
+        <v>5</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I14" s="1">
+        <v>10</v>
+      </c>
+      <c r="J14" s="1">
+        <v>4</v>
+      </c>
+      <c r="K14" s="1">
+        <v>4</v>
+      </c>
+      <c r="L14" s="1">
+        <f>I14*J14*K14</f>
+        <v>160</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="N14" s="2">
+        <v>10</v>
+      </c>
+      <c r="O14" s="2">
+        <v>2</v>
+      </c>
+      <c r="P14" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q14" s="2">
+        <f>N14*O14*P14</f>
+        <v>80</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
+      <c r="A15" s="1">
+        <v>4</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I15" s="1">
+        <v>5</v>
+      </c>
+      <c r="J15" s="1">
+        <v>3</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+      <c r="L15" s="1">
+        <f>I15*J15*K15</f>
+        <v>15</v>
+      </c>
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
       <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
+      <c r="Q15" s="2">
+        <f>N15*O15*P15</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
+      <c r="A16" s="1">
+        <v>3</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="I16" s="1">
+        <v>5</v>
+      </c>
+      <c r="J16" s="1">
+        <v>7</v>
+      </c>
+      <c r="K16" s="1">
+        <v>4</v>
+      </c>
+      <c r="L16" s="1">
+        <f>I16*J16*K16</f>
+        <v>140</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="N16" s="2">
+        <v>5</v>
+      </c>
+      <c r="O16" s="2">
+        <v>4</v>
+      </c>
+      <c r="P16" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q16" s="2">
+        <f>N16*O16*P16</f>
+        <v>60</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
+      <c r="A17" s="1">
+        <v>2</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="I17" s="1">
+        <v>5</v>
+      </c>
+      <c r="J17" s="1">
+        <v>5</v>
+      </c>
+      <c r="K17" s="1">
+        <v>2</v>
+      </c>
+      <c r="L17" s="1">
+        <f>I17*J17*K17</f>
+        <v>50</v>
+      </c>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
+      <c r="Q17" s="2">
+        <f>N17*O17*P17</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
+      <c r="A18" s="1">
+        <v>1</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="I18" s="1">
+        <v>5</v>
+      </c>
+      <c r="J18" s="1">
+        <v>6</v>
+      </c>
+      <c r="K18" s="1">
+        <v>2</v>
+      </c>
+      <c r="L18" s="1">
+        <f>I18*J18*K18</f>
+        <v>60</v>
+      </c>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
+      <c r="Q18" s="2">
+        <f>N18*O18*P18</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1"/>

</xml_diff>

<commit_message>
Semaine 3 : arbre de défaillance quantifié (valeur exacte, Birnbaum, Fussell-Vesely)
</commit_message>
<xml_diff>
--- a/sdf-etude-de-cas/AMDEC_alim_secours.xlsx
+++ b/sdf-etude-de-cas/AMDEC_alim_secours.xlsx
@@ -1,7 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
   <workbookPr/>
   <bookViews>
     <workbookView activeTab="0"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="179">
   <si>
     <t>AMDEC - Alimentation de secours des charges critiques</t>
   </si>
@@ -100,7 +99,7 @@
     <t>Refus de démarrage</t>
   </si>
   <si>
-    <t>Manque de carburant</t>
+    <t>Nourrice Vide (Pompe / Vanne de transfert du GE)</t>
   </si>
   <si>
     <t>GE indisponible à la sollicitation</t>
@@ -347,6 +346,75 @@
   </si>
   <si>
     <t>Analyse périodique du carburant</t>
+  </si>
+  <si>
+    <t>Protection du départ (disjoncteur + réglages)</t>
+  </si>
+  <si>
+    <t>Éliminer un court-circuit sur un départ en isolant ce seul départ</t>
+  </si>
+  <si>
+    <t>Refus de déclenchement</t>
+  </si>
+  <si>
+    <t>Blocage mécanique d'un disjoncteur</t>
+  </si>
+  <si>
+    <t>Disjoncteur non déclenché</t>
+  </si>
+  <si>
+    <t>Perte totale du jeu de barres si court-circuit -&gt; charges critiques</t>
+  </si>
+  <si>
+    <t>Essais de déclenchement périodiques (défaillance cachée)</t>
+  </si>
+  <si>
+    <t>Déclenchement non sélectif</t>
+  </si>
+  <si>
+    <t>Courbes temps-courant mal coordonnées</t>
+  </si>
+  <si>
+    <t>Mauvais disjoncteur déclénché</t>
+  </si>
+  <si>
+    <t>Etudes de sélectivité</t>
+  </si>
+  <si>
+    <t>Onduleur (bypass statique)</t>
+  </si>
+  <si>
+    <t>Refus de basculement du bypass</t>
+  </si>
+  <si>
+    <t>Carte de commande défaillante</t>
+  </si>
+  <si>
+    <t>Aucun tant que l'onduleur fonctionne, sinon perte totale de l'alimentation du jeu de barres si perte de sortie onduleur</t>
+  </si>
+  <si>
+    <t>Essai de basculement périodique</t>
+  </si>
+  <si>
+    <t>Cuve Principale (DCC)</t>
+  </si>
+  <si>
+    <t>Fournir du carburant aux GE</t>
+  </si>
+  <si>
+    <t>Niveau insuffisant pour assurer la mission pendant 24h</t>
+  </si>
+  <si>
+    <t>Manque de carburant (remplissager non effectué)</t>
+  </si>
+  <si>
+    <t>Nourrices non réalimentées</t>
+  </si>
+  <si>
+    <t>Arrêt des GE en cours de mission, perte totale de l'alimentation du jeu de barres après batteries</t>
+  </si>
+  <si>
+    <t>Jauge de carburant + alarme carburant vide + Vérification mensuelle du niveau de la cuve</t>
   </si>
   <si>
     <t>Synthèse</t>
@@ -755,7 +823,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -791,6 +859,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -800,7 +892,7 @@
     <xf numFmtId="42" fontId="20" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -912,6 +1004,8 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1089,7 +1183,7 @@
     <tabColor rgb="FF1F3864"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:Q48"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.00390625" customWidth="1"/>
@@ -1110,71 +1204,39 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
     </row>
     <row r="3" ht="7.5" customHeight="1"/>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="44"/>
       <c r="I4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+      <c r="J4" s="43"/>
+      <c r="K4" s="43"/>
+      <c r="L4" s="44"/>
       <c r="M4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
+      <c r="O4" s="43"/>
+      <c r="P4" s="43"/>
+      <c r="Q4" s="44"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="6" t="s">
@@ -2072,167 +2134,385 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" ht="16.5">
-      <c r="A24" s="15" t="s">
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="7">
+        <v>18</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="16" t="s">
+      <c r="C23" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="17">
-        <f>COUNTA(D6:D22)</f>
-        <v>17</v>
-      </c>
-      <c r="F25" s="18" t="s">
+      <c r="D23" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="18"/>
-      <c r="L25" s="18"/>
-      <c r="M25" s="18"/>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="16" t="s">
+      <c r="E23" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="17">
-        <f>COUNTA(M6:M22)</f>
+      <c r="F23" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="I23" s="7">
+        <v>10</v>
+      </c>
+      <c r="J23" s="7">
+        <v>2</v>
+      </c>
+      <c r="K23" s="7">
+        <v>6</v>
+      </c>
+      <c r="L23" s="14">
+        <f>I23*J23*K23</f>
+        <v>120</v>
+      </c>
+      <c r="M23" s="9"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="7"/>
+      <c r="P23" s="7"/>
+      <c r="Q23" s="10" t="str">
+        <f>IF(COUNT(N23:P23)=3,N23*O23*P23,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="7">
+        <v>19</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="I24" s="7">
+        <v>10</v>
+      </c>
+      <c r="J24" s="7">
+        <v>4</v>
+      </c>
+      <c r="K24" s="7">
         <v>7</v>
       </c>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
-      <c r="J26" s="18"/>
-      <c r="K26" s="18"/>
-      <c r="L26" s="18"/>
-      <c r="M26" s="18"/>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="17">
-        <f>MAX(L6:L22)</f>
-        <v>200</v>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="17">
-        <f t="array" ref="E28">MAX(IF(ISNUMBER(Q6:Q22),Q6:Q22,L6:L22))</f>
+      <c r="L24" s="10">
+        <f>I24*J24*K24</f>
+        <v>280</v>
+      </c>
+      <c r="M24" s="9"/>
+      <c r="N24" s="7"/>
+      <c r="O24" s="7"/>
+      <c r="P24" s="7"/>
+      <c r="Q24" s="14" t="str">
+        <f>IF(COUNT(N24:P24)=3,N24*O24*P24,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1">
+      <c r="A25" s="7">
+        <v>20</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="17">
-        <f>COUNTIF(L6:L22,"&gt;="&amp;SeuilCritique)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="17">
-        <f>SUMPRODUCT(ISNUMBER(Q6:Q22)*(N(+Q6:Q22)&gt;=SeuilCritique))+SUMPRODUCT(NOT(ISNUMBER(Q6:Q22))*(L6:L22&gt;=SeuilCritique))</f>
-        <v>0</v>
+      <c r="C25" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="I25" s="7">
+        <v>10</v>
+      </c>
+      <c r="J25" s="7">
+        <v>3</v>
+      </c>
+      <c r="K25" s="7">
+        <v>6</v>
+      </c>
+      <c r="L25" s="14">
+        <f>I25*J25*K25</f>
+        <v>180</v>
+      </c>
+      <c r="M25" s="9"/>
+      <c r="N25" s="7"/>
+      <c r="O25" s="7"/>
+      <c r="P25" s="7"/>
+      <c r="Q25" s="10" t="str">
+        <f>IF(COUNT(N25:P25)=3,N25*O25*P25,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="7">
+        <v>21</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="I26" s="7">
+        <v>10</v>
+      </c>
+      <c r="J26" s="7">
+        <v>3</v>
+      </c>
+      <c r="K26" s="7">
+        <v>1</v>
+      </c>
+      <c r="L26" s="10">
+        <f>I26*J26*K26</f>
+        <v>30</v>
+      </c>
+      <c r="M26" s="9"/>
+      <c r="N26" s="7"/>
+      <c r="O26" s="7"/>
+      <c r="P26" s="7"/>
+      <c r="Q26" s="10" t="str">
+        <f>IF(COUNT(N26:P26)=3,N26*O26*P26,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
+      <c r="P27" s="7"/>
+      <c r="Q27" s="10"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7"/>
+      <c r="B28" s="43"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="43"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="43"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="7"/>
+      <c r="O28" s="7"/>
+      <c r="P28" s="7"/>
+      <c r="Q28" s="10"/>
+    </row>
+    <row r="29" ht="18" customHeight="1"/>
+    <row r="30" ht="18" customHeight="1"/>
+    <row r="31" ht="18" customHeight="1"/>
+    <row r="32" ht="18" customHeight="1"/>
+    <row r="33" ht="18" customHeight="1"/>
+    <row r="34" ht="18" customHeight="1"/>
+    <row r="42" ht="16.5" customHeight="1">
+      <c r="A42" s="15" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="43" ht="69.75" customHeight="1">
+      <c r="A43" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="B43" s="43"/>
+      <c r="C43" s="43"/>
+      <c r="D43" s="44"/>
+      <c r="E43" s="17">
+        <f>COUNTA(D6:D26)</f>
+        <v>21</v>
+      </c>
+      <c r="F43" s="18" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="B44" s="43"/>
+      <c r="C44" s="43"/>
+      <c r="D44" s="44"/>
+      <c r="E44" s="17">
+        <f>COUNTA(M6:M26)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="B45" s="43"/>
+      <c r="C45" s="43"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="17">
+        <f>MAX(L6:L26)</f>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="B46" s="43"/>
+      <c r="C46" s="43"/>
+      <c r="D46" s="44"/>
+      <c r="E46" s="17">
+        <f t="array" ref="E46">MAX(IF(ISNUMBER(Q6:Q26),Q6:Q26,L6:L26))</f>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B47" s="43"/>
+      <c r="C47" s="43"/>
+      <c r="D47" s="44"/>
+      <c r="E47" s="17">
+        <f>COUNTIF(L6:L26,"&gt;="&amp;SeuilCritique)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="B48" s="43"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="44"/>
+      <c r="E48" s="17">
+        <f>SUMPRODUCT(ISNUMBER(Q6:Q26)*(N(+Q6:Q26)&gt;=SeuilCritique))+SUMPRODUCT(NOT(ISNUMBER(Q6:Q26))*(L6:L26&gt;=SeuilCritique))</f>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:Q22"/>
-  <mergeCells count="13">
+  <mergeCells count="21">
+    <mergeCell ref="I4:L4"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A43:D43"/>
     <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="F43:M44"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="N4:Q4"/>
+    <mergeCell ref="F29:M30"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A42:H42"/>
     <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A46:D46"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="I4:L4"/>
-    <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="F25:M26"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A32:D32"/>
   </mergeCells>
-  <conditionalFormatting sqref="L6:L22">
+  <conditionalFormatting sqref="L6:L26">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND(ISNUMBER(L6),L6&gt;=SeuilCritique)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6:L22">
+  <conditionalFormatting sqref="L6:L26">
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>AND(ISNUMBER(L6),L6&gt;=SeuilSurveillance)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6:L22">
+  <conditionalFormatting sqref="L6:L26">
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>ISNUMBER(L6)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q6:Q22">
+  <conditionalFormatting sqref="Q6:Q26">
     <cfRule type="expression" dxfId="0" priority="4">
       <formula>AND(ISNUMBER(Q6),Q6&gt;=SeuilCritique)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q6:Q22">
+  <conditionalFormatting sqref="Q6:Q26">
     <cfRule type="expression" dxfId="1" priority="5">
       <formula>AND(ISNUMBER(Q6),Q6&gt;=SeuilSurveillance)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q6:Q22">
+  <conditionalFormatting sqref="Q6:Q26">
     <cfRule type="expression" dxfId="2" priority="6">
       <formula>ISNUMBER(Q6)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:I22">
+  <conditionalFormatting sqref="I6:I26">
     <cfRule type="expression" dxfId="3" priority="7">
       <formula>I6&gt;=9</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N6:N22">
+  <conditionalFormatting sqref="N6:N26">
     <cfRule type="expression" dxfId="3" priority="8">
       <formula>AND(ISNUMBER(N6),N6&gt;=9)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Cotation" error="Note entière de 1 à 10" sqref="I6:K22 N6:P22">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Cotation" error="Note entière de 1 à 10" sqref="I6:K26 N6:P26">
       <formula1>1</formula1>
       <formula2>10</formula2>
     </dataValidation>
@@ -2265,186 +2545,183 @@
     <col min="8" max="8" width="9.00390625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21.82">
+    <row r="1" ht="21.82" customHeight="1">
       <c r="A1" s="19" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="20" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="21" t="s">
-        <v>119</v>
-      </c>
-      <c r="B4" s="21"/>
+        <v>142</v>
+      </c>
       <c r="D4" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="E4" s="22"/>
+        <v>143</v>
+      </c>
       <c r="G4" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="H4" s="23"/>
+        <v>144</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="24" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="27" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="B6" s="28">
         <v>1</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="G6" s="27" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="27" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="B7" s="29">
         <v>2</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="H7" s="29" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="27" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="G8" s="27" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="H8" s="30" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="27" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>139</v>
+        <v>162</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="H9" s="31" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="27" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="D10" s="27" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="G10" s="27" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
       <c r="H10" s="32" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="13" ht="16.5">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="33" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="34" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="B14" s="35">
         <f>1/6</f>
         <v>0.16666666666666666</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>148</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="34" t="s">
-        <v>149</v>
+        <v>172</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>150</v>
-      </c>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-    </row>
-    <row r="17" ht="16.5">
+        <v>173</v>
+      </c>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="43"/>
+    </row>
+    <row r="17" ht="16.5" customHeight="1">
       <c r="A17" s="33" t="s">
-        <v>151</v>
+        <v>174</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="B18" s="39">
         <v>125</v>
@@ -2452,7 +2729,7 @@
     </row>
     <row r="19">
       <c r="A19" s="40" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="B19" s="39">
         <v>60</v>
@@ -2460,7 +2737,7 @@
     </row>
     <row r="20">
       <c r="A20" s="41" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="B20" s="42" t="str">
         <f>"&lt; "&amp;B19</f>
@@ -2469,14 +2746,14 @@
     </row>
     <row r="21">
       <c r="A21" s="36" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
     <mergeCell ref="B15:E15"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>